<commit_message>
test: align operator bank tests and fixtures
</commit_message>
<xml_diff>
--- a/backend/src/tests/fixtures/sample.xlsx
+++ b/backend/src/tests/fixtures/sample.xlsx
@@ -397,55 +397,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Month</v>
+        <v>Metric</v>
       </c>
       <c r="B1" t="str">
-        <v>Revenue</v>
+        <v>Jan</v>
       </c>
       <c r="C1" t="str">
-        <v>Cost</v>
+        <v>Feb</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Mar</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Jan</v>
+        <v>Revenue</v>
       </c>
       <c r="B2">
         <v>1200</v>
       </c>
       <c r="C2">
-        <v>800</v>
+        <v>1400</v>
+      </c>
+      <c r="D2">
+        <v>1600</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Feb</v>
+        <v>Cost</v>
       </c>
       <c r="B3">
-        <v>1400</v>
+        <v>800</v>
       </c>
       <c r="C3">
         <v>900</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mar</v>
-      </c>
-      <c r="B4">
-        <v>1600</v>
-      </c>
-      <c r="C4">
+      <c r="D3">
         <v>1000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>